<commit_message>
Make the sample identity numbers impossible to belong to anyone
The invented national IDs in tests/samples used governorate code 12,
which is a real one, so the numbers were complete and valid in every
respect -- exactly the sort of fixture that can turn out to match a
living person's identity number once the repository is public.

They now use governorate code 00, which is assigned to nowhere: every
real code is 01 to 35, or 88 for a birth abroad. The numbers keep the
shape the detector has to catch, which is the whole point of the file,
and can belong to nobody.
</commit_message>
<xml_diff>
--- a/tests/samples/edge_cases.xlsx
+++ b/tests/samples/edge_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Projects\contacts manager\tests\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BABE6533-DB01-4DA1-8DEB-4770ECC59CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1968DCE2-2309-407B-B43D-178CEE1867D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="1480" windowWidth="14400" windowHeight="7360" xr2:uid="{E3068829-0F99-4776-891D-47F1A8C96280}"/>
+    <workbookView xWindow="1480" yWindow="1480" windowWidth="14400" windowHeight="7360" xr2:uid="{11535C5F-3D29-4B31-9FCD-C1F19E38BB9E}"/>
   </bookViews>
   <sheets>
     <sheet name="شاذ" sheetId="1" r:id="rId1"/>
@@ -418,7 +418,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAB8A67B-6812-4C3D-A8EA-D220B6FED721}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6E1174B-5D5E-4AB7-B57B-859A378D394D}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>